<commit_message>
Custom Roles spec-recheck: LIVE role-matrix verification (2026-07-20) — SM/SalesRep/TimeClock confirmed, Office corrected to build (WO/PS kept, Invoicing V/E/D), 3 editable-role build-vs-spec gaps flagged
All 11 system roles read live from /api/roles. Office 7/14 spec removal NOT deployed
(non-editable = true default). SrSA/SvcAdv/Technician gaps flagged as possible shared-org
drift (confirm on clean defaults). Final: 240 OK / 21 UPDATE / 8 OPEN-QUESTION.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KxJ6r8gC8PgunqsXMYkKrZ
</commit_message>
<xml_diff>
--- a/build/custom-roles-run/CustomRoles_SpecRecheck_Proposed-Corrections_2026-07-15.xlsx
+++ b/build/custom-roles-run/CustomRoles_SpecRecheck_Proposed-Corrections_2026-07-15.xlsx
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>Label-rename portion WITHDRAWN (build still shows 'View and Manage AP/AR Data', LIVE 2026-07-20); the BEHAVIOURAL correction on this case still stands. See LIVE-LABEL-CHECK-RESULT.md.</t>
+          <t>LIVE-VERIFIED 2026-07-20: Service Manager = WO V/E/D (Delete present), Invoicing V/E (no Delete), Customers full, Full View. Confirms the correction. (AP/AR label build-accurate: 'View and Manage AP/AR Data'.)</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>expected, label</t>
+          <t>expected</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1840,23 +1840,23 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>[expected] The Office User permissions match the expected set per the 7/14 spec update: Work Orders = NONE (no Work Orders access — the Work Orders nav is hidden for Office); Part Sales = NONE; Invoicing &amp; Payments = View/Create &amp; Edit/Delete (BUT a hard-coded rule disables the Create Invoice button for Office on both Work Orders and Part Sales — Office can make payments/deposits/credits but cannot create invoices); Customers full (including Delete); Catalog and Inventory View only; Vendor and Order Management View only; Timesheets View/Create &amp; Edit; Schedule View only; Reports on; Billing Portal on; See Financial Data on; Manage Accounts Payable and Receivable on; Settings on with App Settings, Integrations, Finance, Data Import and View/Manage Wages; View mode Full View. The Office User role is non-editable (lock icon, eye only).
-OPEN QUESTIONS to flag (do not assert a verdict): (1) the spec matrix lists Office Work Order Lines = View while Office Work Orders = none — a spec-internal contradiction (WOL View is supposed to inherit from WO View); confirm with PO. (2) HOW Office makes payments/deposits without being able to create invoices is still open with the PO (SV-7993 comment 73184 unanswered; SV-8345 closed deferring there) — verify the payment path live but treat the exact gating as PO-pending.</t>
+          <t>[expected] The Office User permissions match the expected set (LIVE-observed on the build 2026-07-20; Office is non-editable): Work Orders View; Work Order Lines View (inherited); Part Sales View; Catalog and Inventory View; Vendor and Order Management View; Customers View/Create &amp; Edit/Delete; Invoicing &amp; Payments View/Create &amp; Edit/Delete; Timesheets View/Create &amp; Edit; Schedule View; Reports on; Billing Portal on; See Financial Data on; Manage Accounts Payable and Receivable on; View Part History on; Settings on with App Settings, Service, Integrations, Finance, Data Import and View/Manage Wages; View mode Full View; role is non-editable.
+The ONLY change vs the old case is Invoicing &amp; Payments: View -&gt; View/Create &amp; Edit/Delete (Office gained invoicing Create &amp; Edit + Delete). NOTE: the 7/14 spec update that REMOVES Office's Work Orders and Part Sales access is NOT yet deployed - the build still grants Office Work Orders View and Part Sales View; flag this build-vs-spec gap to dev/PO. The hard-coded 'Office cannot create invoices (but can take payments)' rule is still an open PO item (SV-7993).</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>The 7/14 spec update REDEFINED Office: Work Orders V-&gt;none, Part Sales V-&gt;none, Invoicing V-&gt;V/E/D (with the hard-coded no-Create-Invoice rule). The case still encodes the pre-7/14 Office (WO View, Part Sales View, Invoicing View). This is the single biggest behavioural drift in the recheck. Two spec-internal open items flagged, not silently resolved.</t>
+          <t>LIVE 2026-07-20 (non-editable role = true default): build gives Office WO View + Part Sales View + Invoicing V/E/D. The 7/14 spec removal of Office WO/Part Sales is NOT deployed, so the earlier spec-derived correction (WO none / PS none) was wrong. Only real change from the old case is Invoicing View -&gt; V/E/D.</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Spec change log 7/14 ('Updated Office Role definition') + matrix Office column + 'Office Users Cannot Create Invoices'; SV-7993 (open); SV-8345 (obsolete); spec 6/10 label. LABEL-BATCH.md.</t>
+          <t>LIVE /api/roles Office (2026-07-20); spec 7/14 Office redefinition (NOT deployed); SV-7993 (open). See LIVE-ROLE-VERIFICATION-2026-07-20.md.</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>Label-rename portion WITHDRAWN (build still shows 'View and Manage AP/AR Data', LIVE 2026-07-20); the BEHAVIOURAL correction on this case still stands. See LIVE-LABEL-CHECK-RESULT.md.</t>
+          <t>LIVE-VERIFIED 2026-07-20: Office (non-editable) = WO View, WOL View, PS View, Cat View, Ven View, Cust V/E/D, Invoicing V/E/D, TS V/E, Schedule View, Reports/BillingPortal/SFD/AP-AR/ViewHistory ON, Full, non-editable. 7/14 WO/PS removal NOT deployed.</t>
         </is>
       </c>
       <c r="N17" s="4" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>Label-rename portion WITHDRAWN (build still shows 'View and Manage AP/AR Data', LIVE 2026-07-20); the BEHAVIOURAL correction on this case still stands. See LIVE-LABEL-CHECK-RESULT.md. History toggle NOT in the role editor: LIVE 2026-07-20 the Cross-Cutting Toggles card has exactly TWO toggles (See Financial Data + View and Manage AP/AR Data) and the Parts group has only 3 children. No 'View History Logs' / 'View Part History' editor toggle exists. The viewHistoryLogs capability persists in the backend and gates the inventory 'Part History' view only. See LIVE-LABEL-CHECK-RESULT.md.</t>
+          <t>LIVE-VERIFIED 2026-07-20: Sales Representative = WO View, WOL View, Customers View+Create&amp;Edit, Part Sales View, Reports ON, SFD ON, AP/AR ON, Full View, everything else off. Confirms NOT Reports-only. (Build AP/AR label 'View and Manage AP/AR Data'; History toggle absent.)</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
@@ -2219,7 +2219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2640,6 +2640,196 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>C26497</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26497</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>3548</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Per-Role Verification</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Senior Service Advisor: role permissions match the expected set</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>OPEN-QUESTION</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>UPDATE</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>...See Financial Data on; View and Manage AP/AR Data on...</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Label find-replace 'View and Manage AP/AR Data' -&gt; 'Manage Accounts Payable and Receivable' (confirm live). Permission set matches spec matrix (SrSA).</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Stale toggle label; permission set correct.</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Spec 6/10; matrix SrSA column. LABEL-BATCH.md.</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>LIVE 2026-07-20: Senior Service Advisor has Reports OFF in the build, but spec matrix says Reports ON. SrSA is editable on a SHARED org so this may be tester drift, or a real build gap. CONFIRM on clean defaults before treating the case's 'Reports on' as wrong. Otherwise the SrSA set matches. (AP/AR label build-accurate.)</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>C26498</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26498</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>3548</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Per-Role Verification</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Service Advisor: role permissions match the expected set</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>OPEN-QUESTION</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>UPDATE</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>...See Financial Data on; View and Manage AP/AR Data OFF...</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Label find-replace (confirm live). Permission set matches spec matrix (Svc Advisor): WO V/E, WOL full, Customers V/E, Part Sales V/E, Invoicing full, Reports off, Customer Portal on, AP/AR off, Full View.</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Stale toggle label; permission set correct.</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Spec 6/10; matrix Svc Advisor column. LABEL-BATCH.md.</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>LIVE 2026-07-20: Service Advisor Invoicing is V/E in the build (no Delete), but spec + case say V/E/D. Editable role on a shared org -&gt; possible drift. CONFIRM on clean defaults. (AP/AR label build-accurate.)</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>C26500</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26500</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>3548</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Per-Role Verification</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Technician: role permissions match the expected set</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>OPEN-QUESTION</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>(no wording change) Matches spec matrix (Tech): WO V, WOL V/E, Schedule V, Customers V, Pick Parts on, Tech View, everything else off. No stale label used.</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr"/>
+      <c r="L9" s="4" t="inlineStr"/>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>LIVE 2026-07-20: Technician shows WO Create&amp;Edit, Customers Create&amp;Edit and See Financial Data ON in the build, vs spec WO View / Customers View / SFD off. CLAUDE.md warns the Technician role is DRIFTED on this shared org; WO C&amp;E + SFD ON is a classic drift signature. RE-DERIVE on clean/reset Technician defaults before treating the case as wrong.</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2651,7 +2841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N244"/>
+  <dimension ref="A1:N241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11177,12 +11367,12 @@
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>C26497</t>
+          <t>C26499</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26497</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26499</t>
         </is>
       </c>
       <c r="C190" s="4" t="n">
@@ -11195,7 +11385,7 @@
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t>Senior Service Advisor: role permissions match the expected set</t>
+          <t>Foreman: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F190" s="4" t="inlineStr">
@@ -11215,12 +11405,12 @@
       </c>
       <c r="I190" s="4" t="inlineStr">
         <is>
-          <t>...See Financial Data on; View and Manage AP/AR Data on...</t>
+          <t>...See Financial Data on; View and Manage AP/AR Data off...</t>
         </is>
       </c>
       <c r="J190" s="4" t="inlineStr">
         <is>
-          <t>Label find-replace 'View and Manage AP/AR Data' -&gt; 'Manage Accounts Payable and Receivable' (confirm live). Permission set matches spec matrix (SrSA).</t>
+          <t>Label find-replace (confirm live). Permission set matches spec matrix (Foreman).</t>
         </is>
       </c>
       <c r="K190" s="4" t="inlineStr">
@@ -11230,7 +11420,7 @@
       </c>
       <c r="L190" s="4" t="inlineStr">
         <is>
-          <t>Spec 6/10; matrix SrSA column. LABEL-BATCH.md.</t>
+          <t>Spec 6/10; matrix Foreman column. LABEL-BATCH.md.</t>
         </is>
       </c>
       <c r="M190" s="4" t="inlineStr">
@@ -11247,12 +11437,12 @@
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>C26498</t>
+          <t>C26501</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26498</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26501</t>
         </is>
       </c>
       <c r="C191" s="4" t="n">
@@ -11265,7 +11455,7 @@
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>Service Advisor: role permissions match the expected set</t>
+          <t>Parts Manager: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F191" s="4" t="inlineStr">
@@ -11285,12 +11475,12 @@
       </c>
       <c r="I191" s="4" t="inlineStr">
         <is>
-          <t>...See Financial Data on; View and Manage AP/AR Data OFF...</t>
+          <t>...See Financial Data on; View and Manage AP/AR Data on; Settings limited to Parts, Finance and Data Import...</t>
         </is>
       </c>
       <c r="J191" s="4" t="inlineStr">
         <is>
-          <t>Label find-replace (confirm live). Permission set matches spec matrix (Svc Advisor): WO V/E, WOL full, Customers V/E, Part Sales V/E, Invoicing full, Reports off, Customer Portal on, AP/AR off, Full View.</t>
+          <t>Label find-replace (confirm live). Permission set matches spec matrix (Parts Mgr): WO V/E (no Delete), WOL V/E (no Delete), Customers full, Parts areas full, Invoicing full, Settings sub Parts/Finance/Data Import, Full View.</t>
         </is>
       </c>
       <c r="K191" s="4" t="inlineStr">
@@ -11300,7 +11490,7 @@
       </c>
       <c r="L191" s="4" t="inlineStr">
         <is>
-          <t>Spec 6/10; matrix Svc Advisor column. LABEL-BATCH.md.</t>
+          <t>Spec 6/10; matrix + sub-toggle table Parts Mgr. LABEL-BATCH.md.</t>
         </is>
       </c>
       <c r="M191" s="4" t="inlineStr">
@@ -11317,12 +11507,12 @@
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>C26499</t>
+          <t>C26505</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26499</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26505</t>
         </is>
       </c>
       <c r="C192" s="4" t="n">
@@ -11335,7 +11525,7 @@
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t>Foreman: role permissions match the expected set</t>
+          <t>Time Clock User: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F192" s="4" t="inlineStr">
@@ -11355,12 +11545,12 @@
       </c>
       <c r="I192" s="4" t="inlineStr">
         <is>
-          <t>...See Financial Data on; View and Manage AP/AR Data off...</t>
+          <t>...See Financial Data and View and Manage AP/AR Data all off.</t>
         </is>
       </c>
       <c r="J192" s="4" t="inlineStr">
         <is>
-          <t>Label find-replace (confirm live). Permission set matches spec matrix (Foreman).</t>
+          <t>Label find-replace 'View and Manage AP/AR Data' -&gt; 'Manage Accounts Payable and Receivable' (confirm live). Permission set correct: WO View, Schedule View, Timesheets View only; everything else off; non-editable; View Mode empty.</t>
         </is>
       </c>
       <c r="K192" s="4" t="inlineStr">
@@ -11370,29 +11560,29 @@
       </c>
       <c r="L192" s="4" t="inlineStr">
         <is>
-          <t>Spec 6/10; matrix Foreman column. LABEL-BATCH.md.</t>
+          <t>Spec 6/10; matrix Time Clock column. LABEL-BATCH.md.</t>
         </is>
       </c>
       <c r="M192" s="4" t="inlineStr">
         <is>
-          <t>AP/AR label build-accurate: LIVE 2026-07-20 the build shows 'View and Manage AP/AR Data' (5 observations). Spec 6/10 rename to 'Manage Accounts Payable and Receivable' is NOT deployed — proposed rename WITHDRAWN; keep the case label as-is. Build-vs-spec label gap flagged to dev (see LIVE-LABEL-CHECK-RESULT.md).</t>
+          <t>LIVE-VERIFIED 2026-07-20: Time Clock User = WO View, Schedule View, Timesheets View only; view_mode none; all cross-toggles off; non-editable. Matches the case. (AP/AR label build-accurate.)</t>
         </is>
       </c>
       <c r="N192" s="4" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>C26500</t>
+          <t>C26506</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26500</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26506</t>
         </is>
       </c>
       <c r="C193" s="4" t="n">
@@ -11405,7 +11595,7 @@
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>Technician: role permissions match the expected set</t>
+          <t>Customer portal is on by default only for Service Advisor, Senior Service Advisor, Service Manager and Parts Manager (and Administrator)</t>
         </is>
       </c>
       <c r="F193" s="4" t="inlineStr">
@@ -11422,7 +11612,7 @@
       <c r="I193" s="4" t="inlineStr"/>
       <c r="J193" s="4" t="inlineStr">
         <is>
-          <t>(no wording change) Matches spec matrix (Tech): WO V, WOL V/E, Schedule V, Customers V, Pick Parts on, Tech View, everything else off. No stale label used.</t>
+          <t>(no wording change) Matches spec toggle table + OQ6.</t>
         </is>
       </c>
       <c r="K193" s="4" t="inlineStr"/>
@@ -11433,25 +11623,25 @@
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>C26501</t>
+          <t>C26510</t>
         </is>
       </c>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26501</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26510</t>
         </is>
       </c>
       <c r="C194" s="4" t="n">
-        <v>3548</v>
+        <v>3549</v>
       </c>
       <c r="D194" s="4" t="inlineStr">
         <is>
-          <t>Per-Role Verification</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
-          <t>Parts Manager: role permissions match the expected set</t>
+          <t>Legacy 'Admin / Administrator' users become 'Administrator' after migration</t>
         </is>
       </c>
       <c r="F194" s="4" t="inlineStr">
@@ -11461,67 +11651,39 @@
       </c>
       <c r="G194" s="4" t="inlineStr">
         <is>
-          <t>UPDATE</t>
-        </is>
-      </c>
-      <c r="H194" s="4" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
-      </c>
-      <c r="I194" s="4" t="inlineStr">
-        <is>
-          <t>...See Financial Data on; View and Manage AP/AR Data on; Settings limited to Parts, Finance and Data Import...</t>
-        </is>
-      </c>
-      <c r="J194" s="4" t="inlineStr">
-        <is>
-          <t>Label find-replace (confirm live). Permission set matches spec matrix (Parts Mgr): WO V/E (no Delete), WOL V/E (no Delete), Customers full, Parts areas full, Invoicing full, Settings sub Parts/Finance/Data Import, Full View.</t>
-        </is>
-      </c>
-      <c r="K194" s="4" t="inlineStr">
-        <is>
-          <t>Stale toggle label; permission set correct.</t>
-        </is>
-      </c>
-      <c r="L194" s="4" t="inlineStr">
-        <is>
-          <t>Spec 6/10; matrix + sub-toggle table Parts Mgr. LABEL-BATCH.md.</t>
-        </is>
-      </c>
-      <c r="M194" s="4" t="inlineStr">
-        <is>
-          <t>AP/AR label build-accurate: LIVE 2026-07-20 the build shows 'View and Manage AP/AR Data' (5 observations). Spec 6/10 rename to 'Manage Accounts Payable and Receivable' is NOT deployed — proposed rename WITHDRAWN; keep the case label as-is. Build-vs-spec label gap flagged to dev (see LIVE-LABEL-CHECK-RESULT.md).</t>
-        </is>
-      </c>
-      <c r="N194" s="4" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H194" s="4" t="inlineStr"/>
+      <c r="I194" s="4" t="inlineStr"/>
+      <c r="J194" s="4" t="inlineStr"/>
+      <c r="K194" s="4" t="inlineStr"/>
+      <c r="L194" s="4" t="inlineStr"/>
+      <c r="M194" s="4" t="inlineStr"/>
+      <c r="N194" s="4" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>C26505</t>
+          <t>C26511</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26505</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26511</t>
         </is>
       </c>
       <c r="C195" s="4" t="n">
-        <v>3548</v>
+        <v>3549</v>
       </c>
       <c r="D195" s="4" t="inlineStr">
         <is>
-          <t>Per-Role Verification</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>Time Clock User: role permissions match the expected set</t>
+          <t>Legacy 'Office' users become 'Office User' after migration</t>
         </is>
       </c>
       <c r="F195" s="4" t="inlineStr">
@@ -11531,67 +11693,39 @@
       </c>
       <c r="G195" s="4" t="inlineStr">
         <is>
-          <t>UPDATE</t>
-        </is>
-      </c>
-      <c r="H195" s="4" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
-      </c>
-      <c r="I195" s="4" t="inlineStr">
-        <is>
-          <t>...See Financial Data and View and Manage AP/AR Data all off.</t>
-        </is>
-      </c>
-      <c r="J195" s="4" t="inlineStr">
-        <is>
-          <t>Label find-replace 'View and Manage AP/AR Data' -&gt; 'Manage Accounts Payable and Receivable' (confirm live). Permission set correct: WO View, Schedule View, Timesheets View only; everything else off; non-editable; View Mode empty.</t>
-        </is>
-      </c>
-      <c r="K195" s="4" t="inlineStr">
-        <is>
-          <t>Stale toggle label; permission set correct.</t>
-        </is>
-      </c>
-      <c r="L195" s="4" t="inlineStr">
-        <is>
-          <t>Spec 6/10; matrix Time Clock column. LABEL-BATCH.md.</t>
-        </is>
-      </c>
-      <c r="M195" s="4" t="inlineStr">
-        <is>
-          <t>AP/AR label build-accurate: LIVE 2026-07-20 the build shows 'View and Manage AP/AR Data' (5 observations). Spec 6/10 rename to 'Manage Accounts Payable and Receivable' is NOT deployed — proposed rename WITHDRAWN; keep the case label as-is. Build-vs-spec label gap flagged to dev (see LIVE-LABEL-CHECK-RESULT.md).</t>
-        </is>
-      </c>
-      <c r="N195" s="4" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H195" s="4" t="inlineStr"/>
+      <c r="I195" s="4" t="inlineStr"/>
+      <c r="J195" s="4" t="inlineStr"/>
+      <c r="K195" s="4" t="inlineStr"/>
+      <c r="L195" s="4" t="inlineStr"/>
+      <c r="M195" s="4" t="inlineStr"/>
+      <c r="N195" s="4" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>C26506</t>
+          <t>C26512</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26506</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26512</t>
         </is>
       </c>
       <c r="C196" s="4" t="n">
-        <v>3548</v>
+        <v>3549</v>
       </c>
       <c r="D196" s="4" t="inlineStr">
         <is>
-          <t>Per-Role Verification</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
-          <t>Customer portal is on by default only for Service Advisor, Senior Service Advisor, Service Manager and Parts Manager (and Administrator)</t>
+          <t>Legacy 'Time Clock' users become 'Time Clock User' after migration</t>
         </is>
       </c>
       <c r="F196" s="4" t="inlineStr">
@@ -11606,11 +11740,7 @@
       </c>
       <c r="H196" s="4" t="inlineStr"/>
       <c r="I196" s="4" t="inlineStr"/>
-      <c r="J196" s="4" t="inlineStr">
-        <is>
-          <t>(no wording change) Matches spec toggle table + OQ6.</t>
-        </is>
-      </c>
+      <c r="J196" s="4" t="inlineStr"/>
       <c r="K196" s="4" t="inlineStr"/>
       <c r="L196" s="4" t="inlineStr"/>
       <c r="M196" s="4" t="inlineStr"/>
@@ -11619,12 +11749,12 @@
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>C26510</t>
+          <t>C26513</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26510</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26513</t>
         </is>
       </c>
       <c r="C197" s="4" t="n">
@@ -11637,7 +11767,7 @@
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>Legacy 'Admin / Administrator' users become 'Administrator' after migration</t>
+          <t>Legacy 'Service Manager' users become 'Service Manager' after migration</t>
         </is>
       </c>
       <c r="F197" s="4" t="inlineStr">
@@ -11661,12 +11791,12 @@
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>C26511</t>
+          <t>C26514</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26511</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26514</t>
         </is>
       </c>
       <c r="C198" s="4" t="n">
@@ -11679,7 +11809,7 @@
       </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
-          <t>Legacy 'Office' users become 'Office User' after migration</t>
+          <t>Legacy 'Senior Service Advisor' users become 'Senior Service Advisor' after migration</t>
         </is>
       </c>
       <c r="F198" s="4" t="inlineStr">
@@ -11703,12 +11833,12 @@
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>C26512</t>
+          <t>C26515</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26512</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26515</t>
         </is>
       </c>
       <c r="C199" s="4" t="n">
@@ -11721,7 +11851,7 @@
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>Legacy 'Time Clock' users become 'Time Clock User' after migration</t>
+          <t>Legacy 'Service Advisor' users become 'Service Advisor' after migration</t>
         </is>
       </c>
       <c r="F199" s="4" t="inlineStr">
@@ -11745,12 +11875,12 @@
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>C26513</t>
+          <t>C26516</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26513</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26516</t>
         </is>
       </c>
       <c r="C200" s="4" t="n">
@@ -11763,7 +11893,7 @@
       </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
-          <t>Legacy 'Service Manager' users become 'Service Manager' after migration</t>
+          <t>Legacy 'Foreman' users become 'Foreman' after migration</t>
         </is>
       </c>
       <c r="F200" s="4" t="inlineStr">
@@ -11787,12 +11917,12 @@
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>C26514</t>
+          <t>C26517</t>
         </is>
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26514</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26517</t>
         </is>
       </c>
       <c r="C201" s="4" t="n">
@@ -11805,7 +11935,7 @@
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>Legacy 'Senior Service Advisor' users become 'Senior Service Advisor' after migration</t>
+          <t>Legacy 'Technician' users become 'Technician' after migration</t>
         </is>
       </c>
       <c r="F201" s="4" t="inlineStr">
@@ -11829,12 +11959,12 @@
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>C26515</t>
+          <t>C26518</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26515</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26518</t>
         </is>
       </c>
       <c r="C202" s="4" t="n">
@@ -11847,7 +11977,7 @@
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t>Legacy 'Service Advisor' users become 'Service Advisor' after migration</t>
+          <t>Legacy 'Parts Manager' users become 'Parts Manager' after migration</t>
         </is>
       </c>
       <c r="F202" s="4" t="inlineStr">
@@ -11871,12 +12001,12 @@
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>C26516</t>
+          <t>C26519</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26516</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26519</t>
         </is>
       </c>
       <c r="C203" s="4" t="n">
@@ -11889,7 +12019,7 @@
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
-          <t>Legacy 'Foreman' users become 'Foreman' after migration</t>
+          <t>Legacy 'Parts Tech / Parts Technician' users become 'Parts Technician' after migration</t>
         </is>
       </c>
       <c r="F203" s="4" t="inlineStr">
@@ -11913,12 +12043,12 @@
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>C26517</t>
+          <t>C26520</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26517</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26520</t>
         </is>
       </c>
       <c r="C204" s="4" t="n">
@@ -11931,7 +12061,7 @@
       </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
-          <t>Legacy 'Technician' users become 'Technician' after migration</t>
+          <t>Legacy 'Sales Representative' users become 'Sales Representative' after migration</t>
         </is>
       </c>
       <c r="F204" s="4" t="inlineStr">
@@ -11955,12 +12085,12 @@
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>C26518</t>
+          <t>C26525</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26518</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26525</t>
         </is>
       </c>
       <c r="C205" s="4" t="n">
@@ -11973,7 +12103,7 @@
       </c>
       <c r="E205" s="4" t="inlineStr">
         <is>
-          <t>Legacy 'Parts Manager' users become 'Parts Manager' after migration</t>
+          <t>Changing a user's role logs that user out and forces them to log in again</t>
         </is>
       </c>
       <c r="F205" s="4" t="inlineStr">
@@ -11997,12 +12127,12 @@
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>C26519</t>
+          <t>C27731</t>
         </is>
       </c>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26519</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/27731</t>
         </is>
       </c>
       <c r="C206" s="4" t="n">
@@ -12015,7 +12145,7 @@
       </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
-          <t>Legacy 'Parts Tech / Parts Technician' users become 'Parts Technician' after migration</t>
+          <t>Legacy 'Owner' users become 'Administrator' after migration (Owner merged into Admin)</t>
         </is>
       </c>
       <c r="F206" s="4" t="inlineStr">
@@ -12039,25 +12169,25 @@
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>C26520</t>
+          <t>C26526</t>
         </is>
       </c>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26520</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26526</t>
         </is>
       </c>
       <c r="C207" s="4" t="n">
-        <v>3549</v>
+        <v>3550</v>
       </c>
       <c r="D207" s="4" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Staff Record Settings</t>
         </is>
       </c>
       <c r="E207" s="4" t="inlineStr">
         <is>
-          <t>Legacy 'Sales Representative' users become 'Sales Representative' after migration</t>
+          <t>Whether a technician can be scheduled depends on their department, not their role</t>
         </is>
       </c>
       <c r="F207" s="4" t="inlineStr">
@@ -12081,25 +12211,25 @@
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
-          <t>C26525</t>
+          <t>C26527</t>
         </is>
       </c>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26525</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26527</t>
         </is>
       </c>
       <c r="C208" s="4" t="n">
-        <v>3549</v>
+        <v>3550</v>
       </c>
       <c r="D208" s="4" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Staff Record Settings</t>
         </is>
       </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
-          <t>Changing a user's role logs that user out and forces them to log in again</t>
+          <t>Clocking in on a work order line depends on the per-staff Time Clock setting</t>
         </is>
       </c>
       <c r="F208" s="4" t="inlineStr">
@@ -12123,25 +12253,25 @@
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>C27731</t>
+          <t>C26528</t>
         </is>
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/27731</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26528</t>
         </is>
       </c>
       <c r="C209" s="4" t="n">
-        <v>3549</v>
+        <v>3550</v>
       </c>
       <c r="D209" s="4" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Staff Record Settings</t>
         </is>
       </c>
       <c r="E209" s="4" t="inlineStr">
         <is>
-          <t>Legacy 'Owner' users become 'Administrator' after migration (Owner merged into Admin)</t>
+          <t>The universal clock in / out is available to any active staff member, whatever their role</t>
         </is>
       </c>
       <c r="F209" s="4" t="inlineStr">
@@ -12165,25 +12295,25 @@
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t>C26526</t>
+          <t>C26529</t>
         </is>
       </c>
       <c r="B210" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26526</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26529</t>
         </is>
       </c>
       <c r="C210" s="4" t="n">
-        <v>3550</v>
+        <v>3551</v>
       </c>
       <c r="D210" s="4" t="inlineStr">
         <is>
-          <t>Staff Record Settings</t>
+          <t>QuickBooks / Integrations</t>
         </is>
       </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
-          <t>Whether a technician can be scheduled depends on their department, not their role</t>
+          <t>QuickBooks settings appear under Integrations when the Integrations sub-toggle is ON</t>
         </is>
       </c>
       <c r="F210" s="4" t="inlineStr">
@@ -12198,7 +12328,11 @@
       </c>
       <c r="H210" s="4" t="inlineStr"/>
       <c r="I210" s="4" t="inlineStr"/>
-      <c r="J210" s="4" t="inlineStr"/>
+      <c r="J210" s="4" t="inlineStr">
+        <is>
+          <t>(no wording change) Already correctly reflects ruling #17 (QB under Integrations; relocation cancelled). Section title 'QuickBooks Relocation' (3551) is itself stale — suggest renaming the section, not the case.</t>
+        </is>
+      </c>
       <c r="K210" s="4" t="inlineStr"/>
       <c r="L210" s="4" t="inlineStr"/>
       <c r="M210" s="4" t="inlineStr"/>
@@ -12207,25 +12341,25 @@
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t>C26527</t>
+          <t>C26530</t>
         </is>
       </c>
       <c r="B211" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26527</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26530</t>
         </is>
       </c>
       <c r="C211" s="4" t="n">
-        <v>3550</v>
+        <v>3551</v>
       </c>
       <c r="D211" s="4" t="inlineStr">
         <is>
-          <t>Staff Record Settings</t>
+          <t>QuickBooks / Integrations</t>
         </is>
       </c>
       <c r="E211" s="4" t="inlineStr">
         <is>
-          <t>Clocking in on a work order line depends on the per-staff Time Clock setting</t>
+          <t>QuickBooks settings are hidden when the Integrations sub-toggle is OFF</t>
         </is>
       </c>
       <c r="F211" s="4" t="inlineStr">
@@ -12240,7 +12374,11 @@
       </c>
       <c r="H211" s="4" t="inlineStr"/>
       <c r="I211" s="4" t="inlineStr"/>
-      <c r="J211" s="4" t="inlineStr"/>
+      <c r="J211" s="4" t="inlineStr">
+        <is>
+          <t>(no wording change) Correct per ruling #17.</t>
+        </is>
+      </c>
       <c r="K211" s="4" t="inlineStr"/>
       <c r="L211" s="4" t="inlineStr"/>
       <c r="M211" s="4" t="inlineStr"/>
@@ -12249,25 +12387,25 @@
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t>C26528</t>
+          <t>C26531</t>
         </is>
       </c>
       <c r="B212" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26528</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26531</t>
         </is>
       </c>
       <c r="C212" s="4" t="n">
-        <v>3550</v>
+        <v>3551</v>
       </c>
       <c r="D212" s="4" t="inlineStr">
         <is>
-          <t>Staff Record Settings</t>
+          <t>QuickBooks / Integrations</t>
         </is>
       </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
-          <t>The universal clock in / out is available to any active staff member, whatever their role</t>
+          <t>The Integrations settings section is present and hosts QuickBooks, IBS and Open API</t>
         </is>
       </c>
       <c r="F212" s="4" t="inlineStr">
@@ -12282,7 +12420,11 @@
       </c>
       <c r="H212" s="4" t="inlineStr"/>
       <c r="I212" s="4" t="inlineStr"/>
-      <c r="J212" s="4" t="inlineStr"/>
+      <c r="J212" s="4" t="inlineStr">
+        <is>
+          <t>(no wording change) Correct per ruling #17 (SV-8157; SV-7493 relocation obsolete).</t>
+        </is>
+      </c>
       <c r="K212" s="4" t="inlineStr"/>
       <c r="L212" s="4" t="inlineStr"/>
       <c r="M212" s="4" t="inlineStr"/>
@@ -12291,25 +12433,25 @@
     <row r="213">
       <c r="A213" s="4" t="inlineStr">
         <is>
-          <t>C26529</t>
+          <t>C26532</t>
         </is>
       </c>
       <c r="B213" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26529</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26532</t>
         </is>
       </c>
       <c r="C213" s="4" t="n">
-        <v>3551</v>
+        <v>3552</v>
       </c>
       <c r="D213" s="4" t="inlineStr">
         <is>
-          <t>QuickBooks / Integrations</t>
+          <t>User Feedback Strings</t>
         </is>
       </c>
       <c r="E213" s="4" t="inlineStr">
         <is>
-          <t>QuickBooks settings appear under Integrations when the Integrations sub-toggle is ON</t>
+          <t>Create success message wording</t>
         </is>
       </c>
       <c r="F213" s="4" t="inlineStr">
@@ -12324,11 +12466,7 @@
       </c>
       <c r="H213" s="4" t="inlineStr"/>
       <c r="I213" s="4" t="inlineStr"/>
-      <c r="J213" s="4" t="inlineStr">
-        <is>
-          <t>(no wording change) Already correctly reflects ruling #17 (QB under Integrations; relocation cancelled). Section title 'QuickBooks Relocation' (3551) is itself stale — suggest renaming the section, not the case.</t>
-        </is>
-      </c>
+      <c r="J213" s="4" t="inlineStr"/>
       <c r="K213" s="4" t="inlineStr"/>
       <c r="L213" s="4" t="inlineStr"/>
       <c r="M213" s="4" t="inlineStr"/>
@@ -12337,25 +12475,25 @@
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
         <is>
-          <t>C26530</t>
+          <t>C26533</t>
         </is>
       </c>
       <c r="B214" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26530</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26533</t>
         </is>
       </c>
       <c r="C214" s="4" t="n">
-        <v>3551</v>
+        <v>3552</v>
       </c>
       <c r="D214" s="4" t="inlineStr">
         <is>
-          <t>QuickBooks / Integrations</t>
+          <t>User Feedback Strings</t>
         </is>
       </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
-          <t>QuickBooks settings are hidden when the Integrations sub-toggle is OFF</t>
+          <t>Update success message wording</t>
         </is>
       </c>
       <c r="F214" s="4" t="inlineStr">
@@ -12370,11 +12508,7 @@
       </c>
       <c r="H214" s="4" t="inlineStr"/>
       <c r="I214" s="4" t="inlineStr"/>
-      <c r="J214" s="4" t="inlineStr">
-        <is>
-          <t>(no wording change) Correct per ruling #17.</t>
-        </is>
-      </c>
+      <c r="J214" s="4" t="inlineStr"/>
       <c r="K214" s="4" t="inlineStr"/>
       <c r="L214" s="4" t="inlineStr"/>
       <c r="M214" s="4" t="inlineStr"/>
@@ -12383,25 +12517,25 @@
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t>C26531</t>
+          <t>C26534</t>
         </is>
       </c>
       <c r="B215" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26531</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26534</t>
         </is>
       </c>
       <c r="C215" s="4" t="n">
-        <v>3551</v>
+        <v>3552</v>
       </c>
       <c r="D215" s="4" t="inlineStr">
         <is>
-          <t>QuickBooks / Integrations</t>
+          <t>User Feedback Strings</t>
         </is>
       </c>
       <c r="E215" s="4" t="inlineStr">
         <is>
-          <t>The Integrations settings section is present and hosts QuickBooks, IBS and Open API</t>
+          <t>Deleting a custom role with 0 users shows a confirmation dialog</t>
         </is>
       </c>
       <c r="F215" s="4" t="inlineStr">
@@ -12416,11 +12550,7 @@
       </c>
       <c r="H215" s="4" t="inlineStr"/>
       <c r="I215" s="4" t="inlineStr"/>
-      <c r="J215" s="4" t="inlineStr">
-        <is>
-          <t>(no wording change) Correct per ruling #17 (SV-8157; SV-7493 relocation obsolete).</t>
-        </is>
-      </c>
+      <c r="J215" s="4" t="inlineStr"/>
       <c r="K215" s="4" t="inlineStr"/>
       <c r="L215" s="4" t="inlineStr"/>
       <c r="M215" s="4" t="inlineStr"/>
@@ -12429,12 +12559,12 @@
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
         <is>
-          <t>C26532</t>
+          <t>C26535</t>
         </is>
       </c>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26532</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26535</t>
         </is>
       </c>
       <c r="C216" s="4" t="n">
@@ -12447,7 +12577,7 @@
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
-          <t>Create success message wording</t>
+          <t>Deleting a custom role that has users is blocked</t>
         </is>
       </c>
       <c r="F216" s="4" t="inlineStr">
@@ -12471,12 +12601,12 @@
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>C26533</t>
+          <t>C26536</t>
         </is>
       </c>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26533</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26536</t>
         </is>
       </c>
       <c r="C217" s="4" t="n">
@@ -12489,7 +12619,7 @@
       </c>
       <c r="E217" s="4" t="inlineStr">
         <is>
-          <t>Update success message wording</t>
+          <t>Turning See Financial Data on shows a confirmation dialog</t>
         </is>
       </c>
       <c r="F217" s="4" t="inlineStr">
@@ -12513,12 +12643,12 @@
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
         <is>
-          <t>C26534</t>
+          <t>C26537</t>
         </is>
       </c>
       <c r="B218" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26534</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26537</t>
         </is>
       </c>
       <c r="C218" s="4" t="n">
@@ -12531,7 +12661,7 @@
       </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
-          <t>Deleting a custom role with 0 users shows a confirmation dialog</t>
+          <t>Creating a role with no name is blocked with a required-field error</t>
         </is>
       </c>
       <c r="F218" s="4" t="inlineStr">
@@ -12555,12 +12685,12 @@
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>C26535</t>
+          <t>C26538</t>
         </is>
       </c>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26535</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26538</t>
         </is>
       </c>
       <c r="C219" s="4" t="n">
@@ -12573,7 +12703,7 @@
       </c>
       <c r="E219" s="4" t="inlineStr">
         <is>
-          <t>Deleting a custom role that has users is blocked</t>
+          <t>Creating a role with the same permissions as an existing role shows a 'similar role' warning</t>
         </is>
       </c>
       <c r="F219" s="4" t="inlineStr">
@@ -12588,7 +12718,11 @@
       </c>
       <c r="H219" s="4" t="inlineStr"/>
       <c r="I219" s="4" t="inlineStr"/>
-      <c r="J219" s="4" t="inlineStr"/>
+      <c r="J219" s="4" t="inlineStr">
+        <is>
+          <t>(no wording change) Self-notes the build has no hard duplicate-NAME block — ties to the C26339 open question on name uniqueness.</t>
+        </is>
+      </c>
       <c r="K219" s="4" t="inlineStr"/>
       <c r="L219" s="4" t="inlineStr"/>
       <c r="M219" s="4" t="inlineStr"/>
@@ -12597,12 +12731,12 @@
     <row r="220">
       <c r="A220" s="4" t="inlineStr">
         <is>
-          <t>C26536</t>
+          <t>C26539</t>
         </is>
       </c>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26536</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26539</t>
         </is>
       </c>
       <c r="C220" s="4" t="n">
@@ -12615,7 +12749,7 @@
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>Turning See Financial Data on shows a confirmation dialog</t>
+          <t>Reassigning a staff member's role updates the row with no success message (billing note in the window)</t>
         </is>
       </c>
       <c r="F220" s="4" t="inlineStr">
@@ -12639,25 +12773,25 @@
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
         <is>
-          <t>C26537</t>
+          <t>C26540</t>
         </is>
       </c>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26537</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26540</t>
         </is>
       </c>
       <c r="C221" s="4" t="n">
-        <v>3552</v>
+        <v>3553</v>
       </c>
       <c r="D221" s="4" t="inlineStr">
         <is>
-          <t>User Feedback Strings</t>
+          <t>Cross-Permission Combinations</t>
         </is>
       </c>
       <c r="E221" s="4" t="inlineStr">
         <is>
-          <t>Creating a role with no name is blocked with a required-field error</t>
+          <t>A role with all permissions off blocks the user from every feature</t>
         </is>
       </c>
       <c r="F221" s="4" t="inlineStr">
@@ -12681,25 +12815,25 @@
     <row r="222">
       <c r="A222" s="4" t="inlineStr">
         <is>
-          <t>C26538</t>
+          <t>C26541</t>
         </is>
       </c>
       <c r="B222" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26538</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26541</t>
         </is>
       </c>
       <c r="C222" s="4" t="n">
-        <v>3552</v>
+        <v>3553</v>
       </c>
       <c r="D222" s="4" t="inlineStr">
         <is>
-          <t>User Feedback Strings</t>
+          <t>Cross-Permission Combinations</t>
         </is>
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t>Creating a role with the same permissions as an existing role shows a 'similar role' warning</t>
+          <t>A role with all permissions on behaves like Administrator but is still a custom role</t>
         </is>
       </c>
       <c r="F222" s="4" t="inlineStr">
@@ -12714,11 +12848,7 @@
       </c>
       <c r="H222" s="4" t="inlineStr"/>
       <c r="I222" s="4" t="inlineStr"/>
-      <c r="J222" s="4" t="inlineStr">
-        <is>
-          <t>(no wording change) Self-notes the build has no hard duplicate-NAME block — ties to the C26339 open question on name uniqueness.</t>
-        </is>
-      </c>
+      <c r="J222" s="4" t="inlineStr"/>
       <c r="K222" s="4" t="inlineStr"/>
       <c r="L222" s="4" t="inlineStr"/>
       <c r="M222" s="4" t="inlineStr"/>
@@ -12727,25 +12857,25 @@
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t>C26539</t>
+          <t>C26542</t>
         </is>
       </c>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26539</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26542</t>
         </is>
       </c>
       <c r="C223" s="4" t="n">
-        <v>3552</v>
+        <v>3553</v>
       </c>
       <c r="D223" s="4" t="inlineStr">
         <is>
-          <t>User Feedback Strings</t>
+          <t>Cross-Permission Combinations</t>
         </is>
       </c>
       <c r="E223" s="4" t="inlineStr">
         <is>
-          <t>Reassigning a staff member's role updates the row with no success message (billing note in the window)</t>
+          <t>A system role cannot be deleted</t>
         </is>
       </c>
       <c r="F223" s="4" t="inlineStr">
@@ -12769,12 +12899,12 @@
     <row r="224">
       <c r="A224" s="4" t="inlineStr">
         <is>
-          <t>C26540</t>
+          <t>C26543</t>
         </is>
       </c>
       <c r="B224" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26540</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26543</t>
         </is>
       </c>
       <c r="C224" s="4" t="n">
@@ -12787,7 +12917,7 @@
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>A role with all permissions off blocks the user from every feature</t>
+          <t>Only Office User and Time Clock User are non-editable; every other system role (including Administrator) is editable</t>
         </is>
       </c>
       <c r="F224" s="4" t="inlineStr">
@@ -12802,7 +12932,11 @@
       </c>
       <c r="H224" s="4" t="inlineStr"/>
       <c r="I224" s="4" t="inlineStr"/>
-      <c r="J224" s="4" t="inlineStr"/>
+      <c r="J224" s="4" t="inlineStr">
+        <is>
+          <t>(no wording change) Matches spec Concepts (Office + Time Clock non-editable; Admin editable but cannot lose admin-page access).</t>
+        </is>
+      </c>
       <c r="K224" s="4" t="inlineStr"/>
       <c r="L224" s="4" t="inlineStr"/>
       <c r="M224" s="4" t="inlineStr"/>
@@ -12811,12 +12945,12 @@
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
         <is>
-          <t>C26541</t>
+          <t>C26544</t>
         </is>
       </c>
       <c r="B225" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26541</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26544</t>
         </is>
       </c>
       <c r="C225" s="4" t="n">
@@ -12829,7 +12963,7 @@
       </c>
       <c r="E225" s="4" t="inlineStr">
         <is>
-          <t>A role with all permissions on behaves like Administrator but is still a custom role</t>
+          <t>Being unable to open Customers does not stop a user from picking a customer when creating a work order</t>
         </is>
       </c>
       <c r="F225" s="4" t="inlineStr">
@@ -12844,7 +12978,11 @@
       </c>
       <c r="H225" s="4" t="inlineStr"/>
       <c r="I225" s="4" t="inlineStr"/>
-      <c r="J225" s="4" t="inlineStr"/>
+      <c r="J225" s="4" t="inlineStr">
+        <is>
+          <t>(no wording change) Matches SV-8002 / OQ10 (data access separate from feature access).</t>
+        </is>
+      </c>
       <c r="K225" s="4" t="inlineStr"/>
       <c r="L225" s="4" t="inlineStr"/>
       <c r="M225" s="4" t="inlineStr"/>
@@ -12853,12 +12991,12 @@
     <row r="226">
       <c r="A226" s="4" t="inlineStr">
         <is>
-          <t>C26542</t>
+          <t>C26545</t>
         </is>
       </c>
       <c r="B226" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26542</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26545</t>
         </is>
       </c>
       <c r="C226" s="4" t="n">
@@ -12871,7 +13009,7 @@
       </c>
       <c r="E226" s="4" t="inlineStr">
         <is>
-          <t>A system role cannot be deleted</t>
+          <t>A Page Access toggle that is off overrides the add/edit/delete boxes inside it</t>
         </is>
       </c>
       <c r="F226" s="4" t="inlineStr">
@@ -12895,12 +13033,12 @@
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
         <is>
-          <t>C26543</t>
+          <t>C26548</t>
         </is>
       </c>
       <c r="B227" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26543</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26548</t>
         </is>
       </c>
       <c r="C227" s="4" t="n">
@@ -12913,7 +13051,7 @@
       </c>
       <c r="E227" s="4" t="inlineStr">
         <is>
-          <t>Only Office User and Time Clock User are non-editable; every other system role (including Administrator) is editable</t>
+          <t>View off with Create &amp; Edit on is prevented by the tick-cascade</t>
         </is>
       </c>
       <c r="F227" s="4" t="inlineStr">
@@ -12928,11 +13066,7 @@
       </c>
       <c r="H227" s="4" t="inlineStr"/>
       <c r="I227" s="4" t="inlineStr"/>
-      <c r="J227" s="4" t="inlineStr">
-        <is>
-          <t>(no wording change) Matches spec Concepts (Office + Time Clock non-editable; Admin editable but cannot lose admin-page access).</t>
-        </is>
-      </c>
+      <c r="J227" s="4" t="inlineStr"/>
       <c r="K227" s="4" t="inlineStr"/>
       <c r="L227" s="4" t="inlineStr"/>
       <c r="M227" s="4" t="inlineStr"/>
@@ -12941,12 +13075,12 @@
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
         <is>
-          <t>C26544</t>
+          <t>C26549</t>
         </is>
       </c>
       <c r="B228" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26544</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26549</t>
         </is>
       </c>
       <c r="C228" s="4" t="n">
@@ -12959,7 +13093,7 @@
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>Being unable to open Customers does not stop a user from picking a customer when creating a work order</t>
+          <t>AP/AR OFF hides the sensitive customer fields on both the Edit Customer window and the customer overview</t>
         </is>
       </c>
       <c r="F228" s="4" t="inlineStr">
@@ -12969,30 +13103,54 @@
       </c>
       <c r="G228" s="4" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H228" s="4" t="inlineStr"/>
-      <c r="I228" s="4" t="inlineStr"/>
+          <t>UPDATE</t>
+        </is>
+      </c>
+      <c r="H228" s="4" t="inlineStr">
+        <is>
+          <t>title, label</t>
+        </is>
+      </c>
+      <c r="I228" s="4" t="inlineStr">
+        <is>
+          <t>...View and Manage AP/AR Data OFF ... hidden on the Edit Customer window. They should also be hidden on the customer overview panel — confirm this live...</t>
+        </is>
+      </c>
       <c r="J228" s="4" t="inlineStr">
         <is>
-          <t>(no wording change) Matches SV-8002 / OQ10 (data access separate from feature access).</t>
-        </is>
-      </c>
-      <c r="K228" s="4" t="inlineStr"/>
-      <c r="L228" s="4" t="inlineStr"/>
-      <c r="M228" s="4" t="inlineStr"/>
-      <c r="N228" s="4" t="inlineStr"/>
+          <t>Label find-replace 'View and Manage AP/AR Data' -&gt; 'Manage Accounts Payable and Receivable' throughout (confirm live). Behaviour matches spec §5b + §1d (7 fields hidden on Edit Customer + Customer Overview panel when Manage AP/AR OFF). SV-8104 (overview-panel leak) was closed OBSOLETE, so the overview-panel hiding is expected.</t>
+        </is>
+      </c>
+      <c r="K228" s="4" t="inlineStr">
+        <is>
+          <t>Stale toggle label; behaviour correct.</t>
+        </is>
+      </c>
+      <c r="L228" s="4" t="inlineStr">
+        <is>
+          <t>Spec 6/10; §5b/§1d; SV-8104 (obsolete). LABEL-BATCH.md.</t>
+        </is>
+      </c>
+      <c r="M228" s="4" t="inlineStr">
+        <is>
+          <t>AP/AR label build-accurate: LIVE 2026-07-20 the build shows 'View and Manage AP/AR Data' (5 observations). Spec 6/10 rename to 'Manage Accounts Payable and Receivable' is NOT deployed — proposed rename WITHDRAWN; keep the case label as-is. Build-vs-spec label gap flagged to dev (see LIVE-LABEL-CHECK-RESULT.md).</t>
+        </is>
+      </c>
+      <c r="N228" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
         <is>
-          <t>C26545</t>
+          <t>C26550</t>
         </is>
       </c>
       <c r="B229" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26545</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26550</t>
         </is>
       </c>
       <c r="C229" s="4" t="n">
@@ -13005,7 +13163,7 @@
       </c>
       <c r="E229" s="4" t="inlineStr">
         <is>
-          <t>A Page Access toggle that is off overrides the add/edit/delete boxes inside it</t>
+          <t>The last Administrator cannot be left with zero users</t>
         </is>
       </c>
       <c r="F229" s="4" t="inlineStr">
@@ -13020,7 +13178,11 @@
       </c>
       <c r="H229" s="4" t="inlineStr"/>
       <c r="I229" s="4" t="inlineStr"/>
-      <c r="J229" s="4" t="inlineStr"/>
+      <c r="J229" s="4" t="inlineStr">
+        <is>
+          <t>(no wording change) Product-rule check; self-hedges 'raise as a finding if no such rule'. Relates to open SV-8332 ('Unable to Change Administrator to Non-Administrator Despite Another Administrator Existing') + spec OQ9 — leave as-is, verify live.</t>
+        </is>
+      </c>
       <c r="K229" s="4" t="inlineStr"/>
       <c r="L229" s="4" t="inlineStr"/>
       <c r="M229" s="4" t="inlineStr"/>
@@ -13029,12 +13191,12 @@
     <row r="230">
       <c r="A230" s="4" t="inlineStr">
         <is>
-          <t>C26548</t>
+          <t>C26551</t>
         </is>
       </c>
       <c r="B230" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26548</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26551</t>
         </is>
       </c>
       <c r="C230" s="4" t="n">
@@ -13047,7 +13209,7 @@
       </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
-          <t>View off with Create &amp; Edit on is prevented by the tick-cascade</t>
+          <t>Universal clock in/out works even for a user whose role has (almost) no permissions</t>
         </is>
       </c>
       <c r="F230" s="4" t="inlineStr">
@@ -13071,25 +13233,25 @@
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>C26549</t>
+          <t>C29446</t>
         </is>
       </c>
       <c r="B231" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26549</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29446</t>
         </is>
       </c>
       <c r="C231" s="4" t="n">
-        <v>3553</v>
+        <v>4091</v>
       </c>
       <c r="D231" s="4" t="inlineStr">
         <is>
-          <t>Cross-Permission Combinations</t>
+          <t>API - Time Clock Enforcement</t>
         </is>
       </c>
       <c r="E231" s="4" t="inlineStr">
         <is>
-          <t>AP/AR OFF hides the sensitive customer fields on both the Edit Customer window and the customer overview</t>
+          <t>Time Clock user CAN read Work Orders via API</t>
         </is>
       </c>
       <c r="F231" s="4" t="inlineStr">
@@ -13099,67 +13261,39 @@
       </c>
       <c r="G231" s="4" t="inlineStr">
         <is>
-          <t>UPDATE</t>
-        </is>
-      </c>
-      <c r="H231" s="4" t="inlineStr">
-        <is>
-          <t>title, label</t>
-        </is>
-      </c>
-      <c r="I231" s="4" t="inlineStr">
-        <is>
-          <t>...View and Manage AP/AR Data OFF ... hidden on the Edit Customer window. They should also be hidden on the customer overview panel — confirm this live...</t>
-        </is>
-      </c>
-      <c r="J231" s="4" t="inlineStr">
-        <is>
-          <t>Label find-replace 'View and Manage AP/AR Data' -&gt; 'Manage Accounts Payable and Receivable' throughout (confirm live). Behaviour matches spec §5b + §1d (7 fields hidden on Edit Customer + Customer Overview panel when Manage AP/AR OFF). SV-8104 (overview-panel leak) was closed OBSOLETE, so the overview-panel hiding is expected.</t>
-        </is>
-      </c>
-      <c r="K231" s="4" t="inlineStr">
-        <is>
-          <t>Stale toggle label; behaviour correct.</t>
-        </is>
-      </c>
-      <c r="L231" s="4" t="inlineStr">
-        <is>
-          <t>Spec 6/10; §5b/§1d; SV-8104 (obsolete). LABEL-BATCH.md.</t>
-        </is>
-      </c>
-      <c r="M231" s="4" t="inlineStr">
-        <is>
-          <t>AP/AR label build-accurate: LIVE 2026-07-20 the build shows 'View and Manage AP/AR Data' (5 observations). Spec 6/10 rename to 'Manage Accounts Payable and Receivable' is NOT deployed — proposed rename WITHDRAWN; keep the case label as-is. Build-vs-spec label gap flagged to dev (see LIVE-LABEL-CHECK-RESULT.md).</t>
-        </is>
-      </c>
-      <c r="N231" s="4" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H231" s="4" t="inlineStr"/>
+      <c r="I231" s="4" t="inlineStr"/>
+      <c r="J231" s="4" t="inlineStr"/>
+      <c r="K231" s="4" t="inlineStr"/>
+      <c r="L231" s="4" t="inlineStr"/>
+      <c r="M231" s="4" t="inlineStr"/>
+      <c r="N231" s="4" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
         <is>
-          <t>C26550</t>
+          <t>C29447</t>
         </is>
       </c>
       <c r="B232" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26550</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29447</t>
         </is>
       </c>
       <c r="C232" s="4" t="n">
-        <v>3553</v>
+        <v>4091</v>
       </c>
       <c r="D232" s="4" t="inlineStr">
         <is>
-          <t>Cross-Permission Combinations</t>
+          <t>API - Time Clock Enforcement</t>
         </is>
       </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
-          <t>The last Administrator cannot be left with zero users</t>
+          <t>Time Clock user CAN read the Schedule via API</t>
         </is>
       </c>
       <c r="F232" s="4" t="inlineStr">
@@ -13174,11 +13308,7 @@
       </c>
       <c r="H232" s="4" t="inlineStr"/>
       <c r="I232" s="4" t="inlineStr"/>
-      <c r="J232" s="4" t="inlineStr">
-        <is>
-          <t>(no wording change) Product-rule check; self-hedges 'raise as a finding if no such rule'. Relates to open SV-8332 ('Unable to Change Administrator to Non-Administrator Despite Another Administrator Existing') + spec OQ9 — leave as-is, verify live.</t>
-        </is>
-      </c>
+      <c r="J232" s="4" t="inlineStr"/>
       <c r="K232" s="4" t="inlineStr"/>
       <c r="L232" s="4" t="inlineStr"/>
       <c r="M232" s="4" t="inlineStr"/>
@@ -13187,25 +13317,25 @@
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t>C26551</t>
+          <t>C29448</t>
         </is>
       </c>
       <c r="B233" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26551</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29448</t>
         </is>
       </c>
       <c r="C233" s="4" t="n">
-        <v>3553</v>
+        <v>4091</v>
       </c>
       <c r="D233" s="4" t="inlineStr">
         <is>
-          <t>Cross-Permission Combinations</t>
+          <t>API - Time Clock Enforcement</t>
         </is>
       </c>
       <c r="E233" s="4" t="inlineStr">
         <is>
-          <t>Universal clock in/out works even for a user whose role has (almost) no permissions</t>
+          <t>Time Clock user is blocked from the Parts / Inventory API</t>
         </is>
       </c>
       <c r="F233" s="4" t="inlineStr">
@@ -13229,12 +13359,12 @@
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t>C29446</t>
+          <t>C29449</t>
         </is>
       </c>
       <c r="B234" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29446</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29449</t>
         </is>
       </c>
       <c r="C234" s="4" t="n">
@@ -13247,7 +13377,7 @@
       </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
-          <t>Time Clock user CAN read Work Orders via API</t>
+          <t>Time Clock user is blocked from the Purchase Orders API</t>
         </is>
       </c>
       <c r="F234" s="4" t="inlineStr">
@@ -13271,12 +13401,12 @@
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>C29447</t>
+          <t>C29450</t>
         </is>
       </c>
       <c r="B235" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29447</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29450</t>
         </is>
       </c>
       <c r="C235" s="4" t="n">
@@ -13289,7 +13419,7 @@
       </c>
       <c r="E235" s="4" t="inlineStr">
         <is>
-          <t>Time Clock user CAN read the Schedule via API</t>
+          <t>Time Clock user is blocked from the Customers list API</t>
         </is>
       </c>
       <c r="F235" s="4" t="inlineStr">
@@ -13313,12 +13443,12 @@
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
         <is>
-          <t>C29448</t>
+          <t>C29451</t>
         </is>
       </c>
       <c r="B236" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29448</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29451</t>
         </is>
       </c>
       <c r="C236" s="4" t="n">
@@ -13331,7 +13461,7 @@
       </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
-          <t>Time Clock user is blocked from the Parts / Inventory API</t>
+          <t>Time Clock user is blocked from the Reports (AP Aging) API</t>
         </is>
       </c>
       <c r="F236" s="4" t="inlineStr">
@@ -13355,12 +13485,12 @@
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
         <is>
-          <t>C29449</t>
+          <t>C29452</t>
         </is>
       </c>
       <c r="B237" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29449</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29452</t>
         </is>
       </c>
       <c r="C237" s="4" t="n">
@@ -13373,7 +13503,7 @@
       </c>
       <c r="E237" s="4" t="inlineStr">
         <is>
-          <t>Time Clock user is blocked from the Purchase Orders API</t>
+          <t>Time Clock user is blocked from the Staff and Roles API</t>
         </is>
       </c>
       <c r="F237" s="4" t="inlineStr">
@@ -13397,12 +13527,12 @@
     <row r="238">
       <c r="A238" s="4" t="inlineStr">
         <is>
-          <t>C29450</t>
+          <t>C29453</t>
         </is>
       </c>
       <c r="B238" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29450</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29453</t>
         </is>
       </c>
       <c r="C238" s="4" t="n">
@@ -13415,7 +13545,7 @@
       </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
-          <t>Time Clock user is blocked from the Customers list API</t>
+          <t>Time Clock user is blocked from the Integrations API</t>
         </is>
       </c>
       <c r="F238" s="4" t="inlineStr">
@@ -13439,12 +13569,12 @@
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
         <is>
-          <t>C29451</t>
+          <t>C29454</t>
         </is>
       </c>
       <c r="B239" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29451</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29454</t>
         </is>
       </c>
       <c r="C239" s="4" t="n">
@@ -13457,7 +13587,7 @@
       </c>
       <c r="E239" s="4" t="inlineStr">
         <is>
-          <t>Time Clock user is blocked from the Reports (AP Aging) API</t>
+          <t>Time Clock user is blocked from the Departments API</t>
         </is>
       </c>
       <c r="F239" s="4" t="inlineStr">
@@ -13481,12 +13611,12 @@
     <row r="240">
       <c r="A240" s="4" t="inlineStr">
         <is>
-          <t>C29452</t>
+          <t>C29455</t>
         </is>
       </c>
       <c r="B240" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29452</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29455</t>
         </is>
       </c>
       <c r="C240" s="4" t="n">
@@ -13499,7 +13629,7 @@
       </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
-          <t>Time Clock user is blocked from the Staff and Roles API</t>
+          <t>Time Clock user cannot change organization Settings via API</t>
         </is>
       </c>
       <c r="F240" s="4" t="inlineStr">
@@ -13523,12 +13653,12 @@
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
         <is>
-          <t>C29453</t>
+          <t>C29456</t>
         </is>
       </c>
       <c r="B241" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29453</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29456</t>
         </is>
       </c>
       <c r="C241" s="4" t="n">
@@ -13541,7 +13671,7 @@
       </c>
       <c r="E241" s="4" t="inlineStr">
         <is>
-          <t>Time Clock user is blocked from the Integrations API</t>
+          <t>Time Clock user cannot delete a Customer via API</t>
         </is>
       </c>
       <c r="F241" s="4" t="inlineStr">
@@ -13562,132 +13692,6 @@
       <c r="M241" s="4" t="inlineStr"/>
       <c r="N241" s="4" t="inlineStr"/>
     </row>
-    <row r="242">
-      <c r="A242" s="4" t="inlineStr">
-        <is>
-          <t>C29454</t>
-        </is>
-      </c>
-      <c r="B242" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29454</t>
-        </is>
-      </c>
-      <c r="C242" s="4" t="n">
-        <v>4091</v>
-      </c>
-      <c r="D242" s="4" t="inlineStr">
-        <is>
-          <t>API - Time Clock Enforcement</t>
-        </is>
-      </c>
-      <c r="E242" s="4" t="inlineStr">
-        <is>
-          <t>Time Clock user is blocked from the Departments API</t>
-        </is>
-      </c>
-      <c r="F242" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G242" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H242" s="4" t="inlineStr"/>
-      <c r="I242" s="4" t="inlineStr"/>
-      <c r="J242" s="4" t="inlineStr"/>
-      <c r="K242" s="4" t="inlineStr"/>
-      <c r="L242" s="4" t="inlineStr"/>
-      <c r="M242" s="4" t="inlineStr"/>
-      <c r="N242" s="4" t="inlineStr"/>
-    </row>
-    <row r="243">
-      <c r="A243" s="4" t="inlineStr">
-        <is>
-          <t>C29455</t>
-        </is>
-      </c>
-      <c r="B243" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29455</t>
-        </is>
-      </c>
-      <c r="C243" s="4" t="n">
-        <v>4091</v>
-      </c>
-      <c r="D243" s="4" t="inlineStr">
-        <is>
-          <t>API - Time Clock Enforcement</t>
-        </is>
-      </c>
-      <c r="E243" s="4" t="inlineStr">
-        <is>
-          <t>Time Clock user cannot change organization Settings via API</t>
-        </is>
-      </c>
-      <c r="F243" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G243" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H243" s="4" t="inlineStr"/>
-      <c r="I243" s="4" t="inlineStr"/>
-      <c r="J243" s="4" t="inlineStr"/>
-      <c r="K243" s="4" t="inlineStr"/>
-      <c r="L243" s="4" t="inlineStr"/>
-      <c r="M243" s="4" t="inlineStr"/>
-      <c r="N243" s="4" t="inlineStr"/>
-    </row>
-    <row r="244">
-      <c r="A244" s="4" t="inlineStr">
-        <is>
-          <t>C29456</t>
-        </is>
-      </c>
-      <c r="B244" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29456</t>
-        </is>
-      </c>
-      <c r="C244" s="4" t="n">
-        <v>4091</v>
-      </c>
-      <c r="D244" s="4" t="inlineStr">
-        <is>
-          <t>API - Time Clock Enforcement</t>
-        </is>
-      </c>
-      <c r="E244" s="4" t="inlineStr">
-        <is>
-          <t>Time Clock user cannot delete a Customer via API</t>
-        </is>
-      </c>
-      <c r="F244" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G244" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H244" s="4" t="inlineStr"/>
-      <c r="I244" s="4" t="inlineStr"/>
-      <c r="J244" s="4" t="inlineStr"/>
-      <c r="K244" s="4" t="inlineStr"/>
-      <c r="L244" s="4" t="inlineStr"/>
-      <c r="M244" s="4" t="inlineStr"/>
-      <c r="N244" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>